<commit_message>
feat: release 0.6.0 with MCP analysis, charts and DBF filters
</commit_message>
<xml_diff>
--- a/examples/ventas-demo.xlsx
+++ b/examples/ventas-demo.xlsx
@@ -3,9 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Ventas" sheetId="1" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" r:id="rId2"/>
-    <sheet name="Catalogo" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -67,10 +65,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,17 +399,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I25"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -448,8 +433,8 @@
       <c r="A2" t="str">
         <v>000001</v>
       </c>
-      <c r="B2" s="1">
-        <v>46296.5</v>
+      <c r="B2" t="str">
+        <v>2026-10-01</v>
       </c>
       <c r="C2" t="str">
         <v>Norte</v>
@@ -460,26 +445,25 @@
       <c r="E2" t="str">
         <v>Cuaderno</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="str">
         <v>1</v>
       </c>
-      <c r="G2" s="2">
-        <v>2490.5</v>
-      </c>
-      <c r="H2" s="2">
-        <f>F2*G2</f>
-        <v>2490.5</v>
-      </c>
-      <c r="I2" t="b">
-        <v>0</v>
+      <c r="G2" t="str">
+        <v>2,490.50</v>
+      </c>
+      <c r="H2" t="str">
+        <v>2,490.50</v>
+      </c>
+      <c r="I2" t="str">
+        <v>FALSE</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
         <v>000002</v>
       </c>
-      <c r="B3" s="1">
-        <v>46297.5</v>
+      <c r="B3" t="str">
+        <v>2026-10-02</v>
       </c>
       <c r="C3" t="str">
         <v>Centro</v>
@@ -490,26 +474,25 @@
       <c r="E3" t="str">
         <v>Lápiz</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="str">
         <v>2</v>
       </c>
-      <c r="G3" s="2">
-        <v>590</v>
-      </c>
-      <c r="H3" s="2">
-        <f>F3*G3</f>
-        <v>1180</v>
-      </c>
-      <c r="I3" t="b">
-        <v>1</v>
+      <c r="G3" t="str">
+        <v>590.00</v>
+      </c>
+      <c r="H3" t="str">
+        <v>1,180.00</v>
+      </c>
+      <c r="I3" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>000003</v>
       </c>
-      <c r="B4" s="1">
-        <v>46298.5</v>
+      <c r="B4" t="str">
+        <v>2026-10-03</v>
       </c>
       <c r="C4" t="str">
         <v>Sur</v>
@@ -520,26 +503,25 @@
       <c r="E4" t="str">
         <v>Carpeta</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="str">
         <v>3</v>
       </c>
-      <c r="G4" s="2">
-        <v>1290.75</v>
-      </c>
-      <c r="H4" s="2">
-        <f>F4*G4</f>
-        <v>3872.25</v>
-      </c>
-      <c r="I4" t="b">
-        <v>1</v>
+      <c r="G4" t="str">
+        <v>1,290.75</v>
+      </c>
+      <c r="H4" t="str">
+        <v>3,872.25</v>
+      </c>
+      <c r="I4" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
         <v>000004</v>
       </c>
-      <c r="B5" s="1">
-        <v>46299.5</v>
+      <c r="B5" t="str">
+        <v>2026-10-04</v>
       </c>
       <c r="C5" t="str">
         <v>Norte</v>
@@ -550,26 +532,25 @@
       <c r="E5" t="str">
         <v>Agenda</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="str">
         <v>4</v>
       </c>
-      <c r="G5" s="2">
-        <v>5990</v>
-      </c>
-      <c r="H5" s="2">
-        <f>F5*G5</f>
-        <v>23960</v>
-      </c>
-      <c r="I5" t="b">
-        <v>1</v>
+      <c r="G5" t="str">
+        <v>5,990.00</v>
+      </c>
+      <c r="H5" t="str">
+        <v>23,960.00</v>
+      </c>
+      <c r="I5" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
         <v>000005</v>
       </c>
-      <c r="B6" s="1">
-        <v>46300.5</v>
+      <c r="B6" t="str">
+        <v>2026-10-05</v>
       </c>
       <c r="C6" t="str">
         <v>Centro</v>
@@ -580,26 +561,25 @@
       <c r="E6" t="str">
         <v>Cuaderno</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="str">
         <v>5</v>
       </c>
-      <c r="G6" s="2">
-        <v>2490.5</v>
-      </c>
-      <c r="H6" s="2">
-        <f>F6*G6</f>
-        <v>12452.5</v>
-      </c>
-      <c r="I6" t="b">
-        <v>1</v>
+      <c r="G6" t="str">
+        <v>2,490.50</v>
+      </c>
+      <c r="H6" t="str">
+        <v>12,452.50</v>
+      </c>
+      <c r="I6" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>000006</v>
       </c>
-      <c r="B7" s="1">
-        <v>46301.5</v>
+      <c r="B7" t="str">
+        <v>2026-10-06</v>
       </c>
       <c r="C7" t="str">
         <v>Sur</v>
@@ -610,26 +590,25 @@
       <c r="E7" t="str">
         <v>Lápiz</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="str">
         <v>1</v>
       </c>
-      <c r="G7" s="2">
-        <v>590</v>
-      </c>
-      <c r="H7" s="2">
-        <f>F7*G7</f>
-        <v>590</v>
-      </c>
-      <c r="I7" t="b">
-        <v>1</v>
+      <c r="G7" t="str">
+        <v>590.00</v>
+      </c>
+      <c r="H7" t="str">
+        <v>590.00</v>
+      </c>
+      <c r="I7" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
         <v>000007</v>
       </c>
-      <c r="B8" s="1">
-        <v>46302.5</v>
+      <c r="B8" t="str">
+        <v>2026-10-07</v>
       </c>
       <c r="C8" t="str">
         <v>Norte</v>
@@ -640,26 +619,25 @@
       <c r="E8" t="str">
         <v>Carpeta</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="str">
         <v>-1</v>
       </c>
-      <c r="G8" s="2">
-        <v>1290.75</v>
-      </c>
-      <c r="H8" s="2">
-        <f>F8*G8</f>
-        <v>-1290.75</v>
-      </c>
-      <c r="I8" t="b">
-        <v>1</v>
+      <c r="G8" t="str">
+        <v>1,290.75</v>
+      </c>
+      <c r="H8" t="str">
+        <v>-1,290.75</v>
+      </c>
+      <c r="I8" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
         <v>000008</v>
       </c>
-      <c r="B9" s="1">
-        <v>46303.5</v>
+      <c r="B9" t="str">
+        <v>2026-10-08</v>
       </c>
       <c r="C9" t="str">
         <v>Centro</v>
@@ -670,26 +648,25 @@
       <c r="E9" t="str">
         <v>Agenda</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="str">
         <v>3</v>
       </c>
-      <c r="G9" s="2">
-        <v>5990</v>
-      </c>
-      <c r="H9" s="2">
-        <f>F9*G9</f>
-        <v>17970</v>
-      </c>
-      <c r="I9" t="b">
-        <v>0</v>
+      <c r="G9" t="str">
+        <v>5,990.00</v>
+      </c>
+      <c r="H9" t="str">
+        <v>17,970.00</v>
+      </c>
+      <c r="I9" t="str">
+        <v>FALSE</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
         <v>000009</v>
       </c>
-      <c r="B10" s="1">
-        <v>46304.5</v>
+      <c r="B10" t="str">
+        <v>2026-10-09</v>
       </c>
       <c r="C10" t="str">
         <v>Sur</v>
@@ -700,26 +677,25 @@
       <c r="E10" t="str">
         <v>Cuaderno</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="str">
         <v>4</v>
       </c>
-      <c r="G10" s="2">
-        <v>2490.5</v>
-      </c>
-      <c r="H10" s="2">
-        <f>F10*G10</f>
-        <v>9962</v>
-      </c>
-      <c r="I10" t="b">
-        <v>1</v>
+      <c r="G10" t="str">
+        <v>2,490.50</v>
+      </c>
+      <c r="H10" t="str">
+        <v>9,962.00</v>
+      </c>
+      <c r="I10" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
         <v>000010</v>
       </c>
-      <c r="B11" s="1">
-        <v>46305.5</v>
+      <c r="B11" t="str">
+        <v>2026-10-10</v>
       </c>
       <c r="C11" t="str">
         <v>Norte</v>
@@ -730,26 +706,25 @@
       <c r="E11" t="str">
         <v>Lápiz</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="str">
         <v>5</v>
       </c>
-      <c r="G11" s="2">
-        <v>590</v>
-      </c>
-      <c r="H11" s="2">
-        <f>F11*G11</f>
-        <v>2950</v>
-      </c>
-      <c r="I11" t="b">
-        <v>1</v>
+      <c r="G11" t="str">
+        <v>590.00</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2,950.00</v>
+      </c>
+      <c r="I11" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
         <v>000011</v>
       </c>
-      <c r="B12" s="1">
-        <v>46306.5</v>
+      <c r="B12" t="str">
+        <v>2026-10-11</v>
       </c>
       <c r="C12" t="str">
         <v>Centro</v>
@@ -760,26 +735,25 @@
       <c r="E12" t="str">
         <v>Carpeta</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="str">
         <v>1</v>
       </c>
-      <c r="G12" s="2">
-        <v>1290.75</v>
-      </c>
-      <c r="H12" s="2">
-        <f>F12*G12</f>
-        <v>1290.75</v>
-      </c>
-      <c r="I12" t="b">
-        <v>1</v>
+      <c r="G12" t="str">
+        <v>1,290.75</v>
+      </c>
+      <c r="H12" t="str">
+        <v>1,290.75</v>
+      </c>
+      <c r="I12" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
         <v>000012</v>
       </c>
-      <c r="B13" s="1">
-        <v>46307.5</v>
+      <c r="B13" t="str">
+        <v>2026-10-12</v>
       </c>
       <c r="C13" t="str">
         <v>Sur</v>
@@ -790,26 +764,25 @@
       <c r="E13" t="str">
         <v>Agenda</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="str">
         <v>2</v>
       </c>
-      <c r="G13" s="2">
-        <v>5990</v>
-      </c>
-      <c r="H13" s="2">
-        <f>F13*G13</f>
-        <v>11980</v>
-      </c>
-      <c r="I13" t="b">
-        <v>1</v>
+      <c r="G13" t="str">
+        <v>5,990.00</v>
+      </c>
+      <c r="H13" t="str">
+        <v>11,980.00</v>
+      </c>
+      <c r="I13" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
         <v>000013</v>
       </c>
-      <c r="B14" s="1">
-        <v>46308.5</v>
+      <c r="B14" t="str">
+        <v>2026-10-13</v>
       </c>
       <c r="C14" t="str">
         <v>Norte</v>
@@ -820,26 +793,25 @@
       <c r="E14" t="str">
         <v>Cuaderno</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="str">
         <v>3</v>
       </c>
-      <c r="G14" s="2">
-        <v>2490.5</v>
-      </c>
-      <c r="H14" s="2">
-        <f>F14*G14</f>
-        <v>7471.5</v>
-      </c>
-      <c r="I14" t="b">
-        <v>1</v>
+      <c r="G14" t="str">
+        <v>2,490.50</v>
+      </c>
+      <c r="H14" t="str">
+        <v>7,471.50</v>
+      </c>
+      <c r="I14" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
         <v>000014</v>
       </c>
-      <c r="B15" s="1">
-        <v>46309.5</v>
+      <c r="B15" t="str">
+        <v>2026-10-14</v>
       </c>
       <c r="C15" t="str">
         <v>Centro</v>
@@ -850,26 +822,25 @@
       <c r="E15" t="str">
         <v>Lápiz</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="str">
         <v>4</v>
       </c>
-      <c r="G15" s="2">
-        <v>590</v>
-      </c>
-      <c r="H15" s="2">
-        <f>F15*G15</f>
-        <v>2360</v>
-      </c>
-      <c r="I15" t="b">
-        <v>1</v>
+      <c r="G15" t="str">
+        <v>590.00</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2,360.00</v>
+      </c>
+      <c r="I15" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
         <v>000015</v>
       </c>
-      <c r="B16" s="1">
-        <v>46310.5</v>
+      <c r="B16" t="str">
+        <v>2026-10-15</v>
       </c>
       <c r="C16" t="str">
         <v>Sur</v>
@@ -880,26 +851,25 @@
       <c r="E16" t="str">
         <v>Carpeta</v>
       </c>
-      <c r="F16">
+      <c r="F16" t="str">
         <v>5</v>
       </c>
-      <c r="G16" s="2">
-        <v>1290.75</v>
-      </c>
-      <c r="H16" s="2">
-        <f>F16*G16</f>
-        <v>6453.75</v>
-      </c>
-      <c r="I16" t="b">
-        <v>0</v>
+      <c r="G16" t="str">
+        <v>1,290.75</v>
+      </c>
+      <c r="H16" t="str">
+        <v>6,453.75</v>
+      </c>
+      <c r="I16" t="str">
+        <v>FALSE</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
         <v>000016</v>
       </c>
-      <c r="B17" s="1">
-        <v>46311.5</v>
+      <c r="B17" t="str">
+        <v>2026-10-16</v>
       </c>
       <c r="C17" t="str">
         <v>Norte</v>
@@ -910,26 +880,25 @@
       <c r="E17" t="str">
         <v>Agenda</v>
       </c>
-      <c r="F17">
+      <c r="F17" t="str">
         <v>1</v>
       </c>
-      <c r="G17" s="2">
-        <v>5990</v>
-      </c>
-      <c r="H17" s="2">
-        <f>F17*G17</f>
-        <v>5990</v>
-      </c>
-      <c r="I17" t="b">
-        <v>1</v>
+      <c r="G17" t="str">
+        <v>5,990.00</v>
+      </c>
+      <c r="H17" t="str">
+        <v>5,990.00</v>
+      </c>
+      <c r="I17" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
         <v>000017</v>
       </c>
-      <c r="B18" s="1">
-        <v>46312.5</v>
+      <c r="B18" t="str">
+        <v>2026-10-17</v>
       </c>
       <c r="C18" t="str">
         <v>Centro</v>
@@ -940,26 +909,25 @@
       <c r="E18" t="str">
         <v>Cuaderno</v>
       </c>
-      <c r="F18">
+      <c r="F18" t="str">
         <v>2</v>
       </c>
-      <c r="G18" s="2">
-        <v>2490.5</v>
-      </c>
-      <c r="H18" s="2">
-        <f>F18*G18</f>
-        <v>4981</v>
-      </c>
-      <c r="I18" t="b">
-        <v>1</v>
+      <c r="G18" t="str">
+        <v>2,490.50</v>
+      </c>
+      <c r="H18" t="str">
+        <v>4,981.00</v>
+      </c>
+      <c r="I18" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
         <v>000018</v>
       </c>
-      <c r="B19" s="1">
-        <v>46313.5</v>
+      <c r="B19" t="str">
+        <v>2026-10-18</v>
       </c>
       <c r="C19" t="str">
         <v>Sur</v>
@@ -970,26 +938,25 @@
       <c r="E19" t="str">
         <v>Lápiz</v>
       </c>
-      <c r="F19">
+      <c r="F19" t="str">
         <v>-1</v>
       </c>
-      <c r="G19" s="2">
-        <v>590</v>
-      </c>
-      <c r="H19" s="2">
-        <f>F19*G19</f>
-        <v>-590</v>
-      </c>
-      <c r="I19" t="b">
-        <v>1</v>
+      <c r="G19" t="str">
+        <v>590.00</v>
+      </c>
+      <c r="H19" t="str">
+        <v>-590.00</v>
+      </c>
+      <c r="I19" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
         <v>000019</v>
       </c>
-      <c r="B20" s="1">
-        <v>46314.5</v>
+      <c r="B20" t="str">
+        <v>2026-10-19</v>
       </c>
       <c r="C20" t="str">
         <v>Norte</v>
@@ -1000,26 +967,25 @@
       <c r="E20" t="str">
         <v>Carpeta</v>
       </c>
-      <c r="F20">
+      <c r="F20" t="str">
         <v>4</v>
       </c>
-      <c r="G20" s="2">
-        <v>1290.75</v>
-      </c>
-      <c r="H20" s="2">
-        <f>F20*G20</f>
-        <v>5163</v>
-      </c>
-      <c r="I20" t="b">
-        <v>1</v>
+      <c r="G20" t="str">
+        <v>1,290.75</v>
+      </c>
+      <c r="H20" t="str">
+        <v>5,163.00</v>
+      </c>
+      <c r="I20" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
         <v>000020</v>
       </c>
-      <c r="B21" s="1">
-        <v>46315.5</v>
+      <c r="B21" t="str">
+        <v>2026-10-20</v>
       </c>
       <c r="C21" t="str">
         <v>Centro</v>
@@ -1030,26 +996,25 @@
       <c r="E21" t="str">
         <v>Agenda</v>
       </c>
-      <c r="F21">
+      <c r="F21" t="str">
         <v>5</v>
       </c>
-      <c r="G21" s="2">
-        <v>5990</v>
-      </c>
-      <c r="H21" s="2">
-        <f>F21*G21</f>
-        <v>29950</v>
-      </c>
-      <c r="I21" t="b">
-        <v>1</v>
+      <c r="G21" t="str">
+        <v>5,990.00</v>
+      </c>
+      <c r="H21" t="str">
+        <v>29,950.00</v>
+      </c>
+      <c r="I21" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
         <v>000021</v>
       </c>
-      <c r="B22" s="1">
-        <v>46316.5</v>
+      <c r="B22" t="str">
+        <v>2026-10-21</v>
       </c>
       <c r="C22" t="str">
         <v>Sur</v>
@@ -1060,26 +1025,25 @@
       <c r="E22" t="str">
         <v>Cuaderno</v>
       </c>
-      <c r="F22">
+      <c r="F22" t="str">
         <v>1</v>
       </c>
-      <c r="G22" s="2">
-        <v>2490.5</v>
-      </c>
-      <c r="H22" s="2">
-        <f>F22*G22</f>
-        <v>2490.5</v>
-      </c>
-      <c r="I22" t="b">
-        <v>1</v>
+      <c r="G22" t="str">
+        <v>2,490.50</v>
+      </c>
+      <c r="H22" t="str">
+        <v>2,490.50</v>
+      </c>
+      <c r="I22" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
         <v>000022</v>
       </c>
-      <c r="B23" s="1">
-        <v>46317.5</v>
+      <c r="B23" t="str">
+        <v>2026-10-22</v>
       </c>
       <c r="C23" t="str">
         <v>Norte</v>
@@ -1090,26 +1054,25 @@
       <c r="E23" t="str">
         <v>Lápiz</v>
       </c>
-      <c r="F23">
+      <c r="F23" t="str">
         <v>2</v>
       </c>
-      <c r="G23" s="2">
-        <v>590</v>
-      </c>
-      <c r="H23" s="2">
-        <f>F23*G23</f>
-        <v>1180</v>
-      </c>
-      <c r="I23" t="b">
-        <v>0</v>
+      <c r="G23" t="str">
+        <v>590.00</v>
+      </c>
+      <c r="H23" t="str">
+        <v>1,180.00</v>
+      </c>
+      <c r="I23" t="str">
+        <v>FALSE</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
         <v>000023</v>
       </c>
-      <c r="B24" s="1">
-        <v>46318.5</v>
+      <c r="B24" t="str">
+        <v>2026-10-23</v>
       </c>
       <c r="C24" t="str">
         <v>Centro</v>
@@ -1120,26 +1083,25 @@
       <c r="E24" t="str">
         <v>Carpeta</v>
       </c>
-      <c r="F24">
+      <c r="F24" t="str">
         <v>3</v>
       </c>
-      <c r="G24" s="2">
-        <v>1290.75</v>
-      </c>
-      <c r="H24" s="2">
-        <f>F24*G24</f>
-        <v>3872.25</v>
-      </c>
-      <c r="I24" t="b">
-        <v>1</v>
+      <c r="G24" t="str">
+        <v>1,290.75</v>
+      </c>
+      <c r="H24" t="str">
+        <v>3,872.25</v>
+      </c>
+      <c r="I24" t="str">
+        <v>TRUE</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
         <v>000024</v>
       </c>
-      <c r="B25" s="1">
-        <v>46319.5</v>
+      <c r="B25" t="str">
+        <v>2026-10-24</v>
       </c>
       <c r="C25" t="str">
         <v>Sur</v>
@@ -1150,18 +1112,17 @@
       <c r="E25" t="str">
         <v>Agenda</v>
       </c>
-      <c r="F25">
+      <c r="F25" t="str">
         <v>4</v>
       </c>
-      <c r="G25" s="2">
-        <v>5990</v>
-      </c>
-      <c r="H25" s="2">
-        <f>F25*G25</f>
-        <v>23960</v>
-      </c>
-      <c r="I25" t="b">
-        <v>1</v>
+      <c r="G25" t="str">
+        <v>5,990.00</v>
+      </c>
+      <c r="H25" t="str">
+        <v>23,960.00</v>
+      </c>
+      <c r="I25" t="str">
+        <v>TRUE</v>
       </c>
     </row>
   </sheetData>
@@ -1169,114 +1130,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:I25"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>REGION</v>
-      </c>
-      <c r="B1" t="str">
-        <v>TOTAL</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Norte</v>
-      </c>
-      <c r="B2" s="2">
-        <f>SUMIF(Ventas!C2:C25,A2,Ventas!H2:H25)</f>
-        <v>47914.25</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Centro</v>
-      </c>
-      <c r="B3" s="2">
-        <f>SUMIF(Ventas!C2:C25,A3,Ventas!H2:H25)</f>
-        <v>74056.5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Sur</v>
-      </c>
-      <c r="B4" s="2">
-        <f>SUMIF(Ventas!C2:C25,A4,Ventas!H2:H25)</f>
-        <v>58718.5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Total general</v>
-      </c>
-      <c r="B5" s="2">
-        <f>SUM(Ventas!H2:H25)</f>
-        <v>180689.25</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>PRODUCTO</v>
-      </c>
-      <c r="B1" t="str">
-        <v>PRECIO</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Cuaderno</v>
-      </c>
-      <c r="B2">
-        <v>2490.5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Lápiz</v>
-      </c>
-      <c r="B3">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Carpeta</v>
-      </c>
-      <c r="B4">
-        <v>1290.75</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Agenda</v>
-      </c>
-      <c r="B5">
-        <v>5990</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>